<commit_message>
docs updated with final test results, signing and build sizes
</commit_message>
<xml_diff>
--- a/docs/TESTING.xlsx
+++ b/docs/TESTING.xlsx
@@ -3374,7 +3374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3792,12 +3792,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>(confirm commit id with the author)</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Fixed (verify)</t>
+          <t>42ee149</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Per-user rules from firestore.rules deployed by the project owner on &lt;date to be confirmed&gt;</t>
+          <t>Per-user rules from firestore.rules deployed with `firebase deploy --only firestore:rules` on 2026-10-21. Before deploying, 4115 allow/deny cases built from every real document were checked with the Firebase rules testing API (owner allowed, other users and signed-out denied) and all passed; then the web app was loaded cold and a write synced</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -3827,9 +3827,9 @@
           <t>(deployment, no commit)</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Fixed (verify)</t>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3841,27 +3841,219 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Unit test for cached written advice fails</t>
+          <t>Unit test for cached written advice failed</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Test still expects the cache key finance_2026-10_... but BUG-10 added the v2_ prefix</t>
+          <t>Test expected the cache key finance_2026-10_... but BUG-10 added the v2_ prefix</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Update the expected key in test/domain/insights/finance_suggestions_test.dart (line 274)</t>
+          <t>Expected key updated in test/domain/insights/finance_suggestions_test.dart</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>6f3cdb3</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>BUG-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>A few tests failed at random in full runs</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Controllers read device storage on start and the tests had no mock, so a MissingPluginException arrived after a test finished; the error reporter then crashed on a stack-trace assertion and hid the cause</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>test/flutter_test_config.dart mocks SharedPreferences and demangles stack traces</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>6f3cdb3</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>BUG-16</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Finance accepted a transaction while signed out (guest-user id)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>A recent change made the user id fall back to guest-user</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Empty id restored so it says "Sign in to save this." and writes nothing; sample data refuses when signed out</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>(code-fix branch)</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>BUG-17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Sync showed Syncing for minutes after loading sample data</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Queued writes were uploaded one at a time, each in its own transaction</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Uploads now go in parallel chunks, one transaction per chunk, order per document kept</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>4d5b5e4</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>BUG-18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Microphone button covered the start of list rows; tile counts flashed 0</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Floating button over content; counts shown before first load</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Mic has its own strip; counts show a dash until the first load finishes</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>(code-fix branch)</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>BUG-19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Wellness water showed 0 ml while Pulse showed 500 ml</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Two separate stores</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Wellness reads and writes the Pulse water events</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>(code-fix branch)</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>BUG-20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Event creation after 11 PM failed validation</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Default end time wrapped to 00:00</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>End clamped to 23:59</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>595254d</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>

</xml_diff>